<commit_message>
fix(client-dash): sheet_source — drop dead code, bounds-safe ts, untagged test
Remove unused _hdr_map(); replace direct index timestamp access with _get()
helper for both LinkedIn and Email blocks; add blank-sentiment reply row to
fixture and assert ReplyRecord.sentiment == "untagged" for blank input.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/client/fixtures/upsta_mini.xlsx
+++ b/tests/client/fixtures/upsta_mini.xlsx
@@ -964,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1168,100 +1168,192 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>reply</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Beta Inc</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/janesmith</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/company/beta</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Jane Smith</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CFO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://linkedin.com/in/sender</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Upsta_US_PMP_V1</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>46184.41666666666</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Tell me more</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>11-50</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Suspect</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Event Type</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Profile Url</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Company Url</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Prospect Name</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Sender Profile</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Date Extraction</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Connection request sent date</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Connection Accepted Date</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Reply Date</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Reply Messages</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Company Country</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Variant</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Reply Sentiment</t>
         </is>

</xml_diff>